<commit_message>
Weekly data update: 2026-09-24, Pre-General filing data
- Re-scraped 452 state filing summaries with 42-Day Pre-General period
- Updated FEC receipts (269K rows) and expenditures
- R aggregation with fresh filing overlay (423 candidates)
- Re-added write-in candidates to state CSV
- Updated footer dates on all 6 pages
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -575,7 +575,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>jonathan bush</t>
+          <t>hannah pingree</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -585,11 +585,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
-        <v>3217769.65</v>
+        <v>4303511.41</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -600,7 +600,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>hannah pingree</t>
+          <t>jonathan bush</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -610,11 +610,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>3039523.78</v>
+        <v>3217769.65</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -675,7 +675,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>nirav shah</t>
+          <t>robert b charles</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -685,11 +685,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E6">
-        <v>1476415.96</v>
+        <v>1842166.4</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -700,7 +700,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>robert b charles</t>
+          <t>nirav shah</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -710,11 +710,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E7">
-        <v>1334066.66</v>
+        <v>1476415.96</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="E10">
-        <v>781017.95</v>
+        <v>926997.04</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1092,7 +1092,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>barbara anne bagshaw</t>
+          <t>bradley youngs</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1105,11 +1105,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
-        <v>1000</v>
+        <v>1003.75</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1120,7 +1120,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>bradley youngs</t>
+          <t>barbara anne bagshaw</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>993.59</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1333,7 +1333,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1000.66</v>
+        <v>1002.32</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1431,7 +1431,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3228.75</v>
+        <v>4728.75</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4805</v>
+        <v>7240.15</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>9833.75</v>
+        <v>13653.75</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1851,7 +1851,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1386.18</v>
+        <v>2482.7</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1879,7 +1879,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1949,7 +1949,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>12371.1</v>
+        <v>16298.74</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2212,7 +2212,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>donald james ardell</t>
+          <t>melanie ann tompkins</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2225,11 +2225,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
-        <v>146.23</v>
+        <v>400</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2240,7 +2240,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>melanie ann tompkins</t>
+          <t>donald james ardell</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2253,11 +2253,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>146.23</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>13301.02</v>
+        <v>15801.53</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2621,7 +2621,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>8733.43</v>
+        <v>9733.43</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2719,7 +2719,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>12967.43</v>
+        <v>17167.43</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2747,7 +2747,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>945.03</v>
+        <v>945.23</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2817,7 +2817,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4050.01</v>
+        <v>8948.379999999999</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2943,7 +2943,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>330.52</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3139,7 +3139,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5106</v>
+        <v>11060.7</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3167,7 +3167,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1000.08</v>
+        <v>1000.3</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3237,7 +3237,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5022.09</v>
+        <v>6022.09</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3318,7 +3318,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>jessica bonafine blanchard</t>
+          <t>dean a cray</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3331,11 +3331,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>2210.03</v>
+        <v>4198.5</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3346,7 +3346,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>dean a cray</t>
+          <t>jessica bonafine blanchard</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3359,11 +3359,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>2198.5</v>
+        <v>2260.03</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3433,7 +3433,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>11200</v>
+        <v>12200</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3531,7 +3531,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4408.48</v>
+        <v>6408.5</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3629,7 +3629,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3134.46</v>
+        <v>4634.46</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3727,7 +3727,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>8116.7</v>
+        <v>9616.719999999999</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3853,7 +3853,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>819.47</v>
+        <v>800</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4975</v>
+        <v>5975</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4049,7 +4049,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1480</v>
+        <v>2025</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4147,7 +4147,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>26355.95</v>
+        <v>31289.48</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4175,7 +4175,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>7900</v>
+        <v>10150</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4497,7 +4497,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3574.58</v>
+        <v>7324.58</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4595,7 +4595,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>9136.700000000001</v>
+        <v>14046.7</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4693,7 +4693,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1250</v>
+        <v>2250</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4791,7 +4791,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2450</v>
+        <v>4660</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4987,7 +4987,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4551.57</v>
+        <v>6251.57</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5183,7 +5183,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2254.58</v>
+        <v>6733.88</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5264,7 +5264,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>mark walker</t>
+          <t>cassandra anne dove</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -5277,11 +5277,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
-        <v>1000</v>
+        <v>1215</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5292,7 +5292,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>cassandra anne dove</t>
+          <t>mark walker</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5305,11 +5305,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>250</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -5505,7 +5505,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3464.7</v>
+        <v>12372.43</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5603,7 +5603,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>15721.07</v>
+        <v>15821.07</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5701,7 +5701,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>250</v>
+        <v>2220</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5799,7 +5799,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6155.59</v>
+        <v>7605.59</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5897,7 +5897,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>18411.5</v>
+        <v>19930.9</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5925,7 +5925,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>251.25</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -5995,7 +5995,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2705.29</v>
+        <v>4605.29</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6219,7 +6219,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>8155.22</v>
+        <v>8156.14</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6317,7 +6317,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3000</v>
+        <v>6000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6345,7 +6345,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>285.35</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -6541,7 +6541,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>11203.6</v>
+        <v>17005.6</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6639,7 +6639,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>56622.02</v>
+        <v>60277.02</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6748,7 +6748,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>kerryl lee clement</t>
+          <t>luke jensen</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6761,7 +6761,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
@@ -6776,7 +6776,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>luke jensen</t>
+          <t>kerryl lee clement</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6789,11 +6789,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>1000</v>
+        <v>900</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -6961,7 +6961,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>1200.03</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -7605,7 +7605,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4500</v>
+        <v>5135</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -7829,7 +7829,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>17727.06</v>
+        <v>34645.74</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -7857,7 +7857,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>13069.13</v>
+        <v>20982.18</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8193,7 +8193,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3858.5</v>
+        <v>6658.71</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8319,7 +8319,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>12217.32</v>
+        <v>15717.32</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8417,7 +8417,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>7299</v>
+        <v>7799</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8445,7 +8445,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>5100</v>
+        <v>7300</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8554,7 +8554,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>harold hull</t>
+          <t>janel c underwoodcharette</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -8571,7 +8571,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>1644</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8582,7 +8582,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>janel c underwoodcharette</t>
+          <t>harold hull</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -8767,7 +8767,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>28964.01</v>
+        <v>46854.01</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8974,7 +8974,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>matthea elisabeth larsen daughtry</t>
+          <t>bernard robert porter</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8987,11 +8987,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>2723.1</v>
+        <v>7285</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9002,7 +9002,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>bernard robert porter</t>
+          <t>matthea elisabeth larsen daughtry</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -9015,11 +9015,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>2395</v>
+        <v>2723.1</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -9327,7 +9327,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>40100</v>
+        <v>46475</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9593,7 +9593,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>23200</v>
+        <v>63943.6</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9691,7 +9691,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>17863.07</v>
+        <v>24742.55</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9747,7 +9747,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>2750</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -9901,7 +9901,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>2149.44</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -10125,7 +10125,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5910.49</v>
+        <v>8710.49</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10223,7 +10223,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>22430.52</v>
+        <v>30465.52</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10643,7 +10643,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>8524.84</v>
+        <v>10174.84</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10923,7 +10923,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>25620</v>
+        <v>29280</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11343,7 +11343,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>871</v>
+        <v>1041</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11413,7 +11413,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>28102.13</v>
+        <v>29173.13</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11441,7 +11441,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -11539,7 +11539,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3765</v>
+        <v>3915</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11917,7 +11917,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1600</v>
+        <v>3765</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12015,7 +12015,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>38677.31</v>
+        <v>39748.19</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12096,7 +12096,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>robert cameron</t>
+          <t>lucy louisa perkins</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -12113,7 +12113,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>952.55</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12124,7 +12124,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>lucy louisa perkins</t>
+          <t>robert cameron</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -12407,7 +12407,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4865.4</v>
+        <v>7446.32</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12729,7 +12729,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6441.46</v>
+        <v>10517.81</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12880,7 +12880,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>suzanne m salisbury</t>
+          <t>lawrence mcwilliams</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -12893,11 +12893,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Unenrolled</t>
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>4822.4</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12908,7 +12908,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>lawrence mcwilliams</t>
+          <t>suzanne m salisbury</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -12921,7 +12921,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
@@ -13261,7 +13261,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5000</v>
+        <v>15000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13527,7 +13527,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>11166.16</v>
+        <v>14341.16</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13555,7 +13555,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>671.76</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -13625,7 +13625,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3676</v>
+        <v>6326</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13751,7 +13751,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>947.02</v>
+        <v>947.1</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -13849,7 +13849,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6700</v>
+        <v>7340.58</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14045,7 +14045,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5900</v>
+        <v>7110</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14143,7 +14143,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2975</v>
+        <v>9325</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14339,7 +14339,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>21819.2</v>
+        <v>24349.29</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14437,7 +14437,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>7084.73</v>
+        <v>13033.73</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14465,7 +14465,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1000.98</v>
+        <v>1029.65</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -14591,7 +14591,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>80</v>
+        <v>230</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14672,7 +14672,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ayn hanselmann</t>
+          <t>domingo e torres</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -14685,11 +14685,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>1000</v>
+        <v>4900</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14700,7 +14700,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>domingo e torres</t>
+          <t>ayn hanselmann</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -14713,11 +14713,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -14798,7 +14798,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>eric h small</t>
+          <t>melissa a simpson</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -14815,7 +14815,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3000.04</v>
+        <v>3450</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14826,7 +14826,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>john robert henkelman iii</t>
+          <t>eric h small</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -14839,11 +14839,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>1000</v>
+        <v>3000.04</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -14854,7 +14854,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>melissa a simpson</t>
+          <t>john robert henkelman iii</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -14867,11 +14867,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -14924,7 +14924,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>jeff adams</t>
+          <t>karen a gerrish</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -14941,7 +14941,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>371.49</v>
+        <v>6763.64</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14952,7 +14952,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>corinna cole</t>
+          <t>jeff adams</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -14965,11 +14965,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>50</v>
+        <v>371.49</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -14980,7 +14980,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>karen a gerrish</t>
+          <t>corinna cole</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -14993,11 +14993,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Unenrolled</t>
         </is>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -15333,7 +15333,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3509.36</v>
+        <v>4009.36</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15487,7 +15487,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3400</v>
+        <v>8035</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15596,7 +15596,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>holly rae eaton</t>
+          <t>clifford noyes</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -15609,11 +15609,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Unenrolled</t>
         </is>
       </c>
       <c r="E2">
-        <v>530</v>
+        <v>1600</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15624,7 +15624,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>clifford noyes</t>
+          <t>holly rae eaton</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -15637,11 +15637,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>533</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -15809,7 +15809,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3229.7</v>
+        <v>4009.7</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15907,7 +15907,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1600</v>
+        <v>2400</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -16131,7 +16131,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>15929.56</v>
+        <v>18529.56</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -16159,7 +16159,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>16312.5</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -16229,7 +16229,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3000</v>
+        <v>3500</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -16425,7 +16425,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1500</v>
+        <v>2500</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -16747,7 +16747,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1299.03</v>
+        <v>1949.03</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -16901,7 +16901,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>725</v>
+        <v>625</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -17248,7 +17248,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>edward l paradis</t>
+          <t>adam shaw</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -17261,11 +17261,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Unenrolled</t>
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>833.3200000000001</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -17276,7 +17276,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>adam shaw</t>
+          <t>edward l paradis</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -17289,7 +17289,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E4">
@@ -17363,7 +17363,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5301.02</v>
+        <v>5701.02</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17461,7 +17461,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1000.01</v>
+        <v>1000.71</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17741,7 +17741,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6100</v>
+        <v>8050</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17867,7 +17867,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2784.51</v>
+        <v>3284.51</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17993,7 +17993,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>600</v>
+        <v>1650</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -18133,7 +18133,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>12731.79</v>
+        <v>18731.79</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18231,7 +18231,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2600.66</v>
+        <v>2700.66</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18427,7 +18427,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>505</v>
+        <v>1835</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18623,7 +18623,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>33840.49</v>
+        <v>39846.35</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18721,7 +18721,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2437.56</v>
+        <v>3637.56</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18847,7 +18847,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3850</v>
+        <v>4850</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19015,7 +19015,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1210</v>
+        <v>1410</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19113,7 +19113,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3070</v>
+        <v>3760</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19337,7 +19337,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1673.46</v>
+        <v>2673.46</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19435,7 +19435,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>9334.469999999999</v>
+        <v>15007.15</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19463,7 +19463,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>5335.5</v>
+        <v>6856.01</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -19589,7 +19589,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>8369.799999999999</v>
+        <v>13942.27</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19715,7 +19715,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>24487</v>
+        <v>27794</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19743,7 +19743,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>5530.13</v>
+        <v>5905.13</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -20261,7 +20261,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>559</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Weekly data update: 2026-10-16, remove Troy Jackson filing note
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -1851,7 +1851,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2482.7</v>
+        <v>2522.7</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5799,7 +5799,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>7605.59</v>
+        <v>8463.889999999999</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6667,7 +6667,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>2551.65</v>
+        <v>7016.65</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8417,7 +8417,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>7799</v>
+        <v>13299</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10755,7 +10755,7 @@
         </is>
       </c>
       <c r="E6">
-        <v>20.18</v>
+        <v>631.29</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -15344,7 +15344,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>margaret wheeler</t>
+          <t>marissa l tasker</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -15361,7 +15361,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -15372,7 +15372,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>marissa l tasker</t>
+          <t>margaret wheeler</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -16327,7 +16327,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>8232.709999999999</v>
+        <v>8332.709999999999</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18623,7 +18623,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>39846.35</v>
+        <v>40305.24</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19743,7 +19743,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>5905.13</v>
+        <v>5969.95</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix ActBlue misattribution bug affecting 46 candidates' top donor lists
The committee_sum logic in clean_state_data.R was misreading transaction
direction — when candidates donated TO ActBlue, the script attributed it
as ActBlue donating to the candidate. Removed the backwards
committee_sum/cand_comm_contribs joins since cand_sum and
cand_contributors already correctly capture all contributions from
candidate filings. Totals were unaffected (filing overlay). Also
refreshes footer dates to October 22 and re-adds write-in candidates.
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -7392,7 +7392,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>kevin oconnell</t>
+          <t>jaric t fontaine</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -7420,7 +7420,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>jaric t fontaine</t>
+          <t>kevin oconnell</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -10402,7 +10402,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>daniel sayre</t>
+          <t>jonathan reed fallon</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -10415,7 +10415,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
@@ -10430,7 +10430,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>jonathan reed fallon</t>
+          <t>daniel sayre</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -10443,7 +10443,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
@@ -12292,7 +12292,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>annie christy</t>
+          <t>michelle n boyer</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -12305,7 +12305,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
@@ -12320,7 +12320,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>michelle n boyer</t>
+          <t>annie christy</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -12333,7 +12333,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">

</xml_diff>

<commit_message>
Weekly state data update: 11-Day Pre-General filings, 332 candidates updated
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4303511.41</v>
+        <v>4978712.13</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -650,7 +650,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>shenna bellows</t>
+          <t>robert b charles</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -660,11 +660,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E5">
-        <v>1910163.56</v>
+        <v>2012008.18</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -675,7 +675,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>robert b charles</t>
+          <t>shenna bellows</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -685,11 +685,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E6">
-        <v>1842166.4</v>
+        <v>1910163.56</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="E10">
-        <v>926997.04</v>
+        <v>964133.28</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="E15">
-        <v>29583.92</v>
+        <v>30401.72</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1109,7 +1109,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1003.75</v>
+        <v>1008.5</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1333,7 +1333,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1002.32</v>
+        <v>1002.97</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1431,7 +1431,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4728.75</v>
+        <v>5228.75</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>7240.15</v>
+        <v>8231.950000000001</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>13653.75</v>
+        <v>17253.75</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1851,7 +1851,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2522.7</v>
+        <v>3947.45</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1879,7 +1879,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1500</v>
+        <v>2811.47</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1949,7 +1949,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>16298.74</v>
+        <v>16805.62</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2229,7 +2229,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>400</v>
+        <v>530</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>15801.53</v>
+        <v>15826.65</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2621,7 +2621,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>9733.43</v>
+        <v>11383.43</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2719,7 +2719,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>17167.43</v>
+        <v>19167.43</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2747,7 +2747,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>945.23</v>
+        <v>945.34</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3139,7 +3139,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>11060.7</v>
+        <v>13473.45</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3167,7 +3167,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1000.3</v>
+        <v>1000.38</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3237,7 +3237,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6022.09</v>
+        <v>8522.09</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3335,7 +3335,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4198.5</v>
+        <v>4248.5</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3433,7 +3433,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>12200</v>
+        <v>13500</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3531,7 +3531,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6408.5</v>
+        <v>7358.52</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3629,7 +3629,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4634.46</v>
+        <v>5284.46</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3727,7 +3727,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>9616.719999999999</v>
+        <v>10091.73</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5975</v>
+        <v>8225</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4049,7 +4049,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2025</v>
+        <v>7632</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4147,7 +4147,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>31289.48</v>
+        <v>32991.98</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4175,7 +4175,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>10150</v>
+        <v>12480</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4497,7 +4497,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>7324.58</v>
+        <v>7574.58</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4693,7 +4693,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2250</v>
+        <v>2850</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4791,7 +4791,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4660</v>
+        <v>4810</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4861,7 +4861,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4720</v>
+        <v>6320</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4987,7 +4987,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6251.57</v>
+        <v>11201.57</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5183,7 +5183,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6733.88</v>
+        <v>10358.88</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5281,7 +5281,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1215</v>
+        <v>2163.21</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5505,7 +5505,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>12372.43</v>
+        <v>15989.73</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5701,7 +5701,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2220</v>
+        <v>2685</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5799,7 +5799,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>8463.889999999999</v>
+        <v>12777.27</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5897,7 +5897,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>19930.9</v>
+        <v>21985.43</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6219,7 +6219,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>8156.14</v>
+        <v>8156.61</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6317,7 +6317,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6000</v>
+        <v>6710</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6541,7 +6541,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>17005.6</v>
+        <v>20080.6</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6639,7 +6639,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>60277.02</v>
+        <v>63182.02</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6667,7 +6667,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>7016.65</v>
+        <v>9766.65</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -6961,7 +6961,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1200.03</v>
+        <v>700.03</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -7605,7 +7605,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5135</v>
+        <v>6635</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -7829,7 +7829,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>34645.74</v>
+        <v>36914.21</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -7857,7 +7857,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>20982.18</v>
+        <v>27860.35</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8193,7 +8193,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6658.71</v>
+        <v>6858.83</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8319,7 +8319,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>15717.32</v>
+        <v>20217.32</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8417,7 +8417,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>13299</v>
+        <v>15949</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8445,7 +8445,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>7300</v>
+        <v>9800</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8767,7 +8767,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>46854.01</v>
+        <v>59359.01</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8991,7 +8991,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>7285</v>
+        <v>7905</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9327,7 +9327,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>46475</v>
+        <v>53975</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9593,7 +9593,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>63943.6</v>
+        <v>69443.60000000001</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9691,7 +9691,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>24742.55</v>
+        <v>26767.55</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10125,7 +10125,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>8710.49</v>
+        <v>11835.49</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10223,7 +10223,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>30465.52</v>
+        <v>33791.52</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10643,7 +10643,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>10174.84</v>
+        <v>11934.54</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10923,7 +10923,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>29280</v>
+        <v>31361</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11343,7 +11343,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1041</v>
+        <v>1051</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11413,7 +11413,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>29173.13</v>
+        <v>30450.13</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11539,7 +11539,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3915</v>
+        <v>3965</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11679,7 +11679,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2895</v>
+        <v>3295</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12015,7 +12015,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>39748.19</v>
+        <v>40558.62</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12729,7 +12729,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>10517.81</v>
+        <v>11778.54</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12897,7 +12897,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4822.4</v>
+        <v>5492.4</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13261,7 +13261,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>15000</v>
+        <v>17000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13359,7 +13359,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1334.25</v>
+        <v>1334.53</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13527,7 +13527,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>14341.16</v>
+        <v>19351.16</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13555,7 +13555,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>671.76</v>
+        <v>4271.76</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -13625,7 +13625,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6326</v>
+        <v>10726</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13751,7 +13751,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>947.1</v>
+        <v>947.24</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -13849,7 +13849,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>7340.58</v>
+        <v>9541.610000000001</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14045,7 +14045,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>7110</v>
+        <v>7710</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14339,7 +14339,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>24349.29</v>
+        <v>24499.29</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14437,7 +14437,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>13033.73</v>
+        <v>14803.73</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14465,7 +14465,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1029.65</v>
+        <v>1000.98</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -14591,7 +14591,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>230</v>
+        <v>628.03</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14689,7 +14689,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4900</v>
+        <v>6700</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14815,7 +14815,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3450</v>
+        <v>9136</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14941,7 +14941,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6763.64</v>
+        <v>8278.17</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15487,7 +15487,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>8035</v>
+        <v>9875</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15613,7 +15613,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1600</v>
+        <v>1800</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15809,7 +15809,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4009.7</v>
+        <v>4400.5</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15907,7 +15907,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2400</v>
+        <v>3000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15988,7 +15988,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>gary gene runnells jr</t>
+          <t>eric white</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -16001,11 +16001,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>2435</v>
+        <v>6100</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -16016,7 +16016,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>nina a milliken</t>
+          <t>gary gene runnells jr</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -16029,11 +16029,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Unenrolled</t>
         </is>
       </c>
       <c r="E3">
-        <v>1000</v>
+        <v>2435</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -16044,7 +16044,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>eric white</t>
+          <t>nina a milliken</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -16057,11 +16057,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -16114,7 +16114,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>steven matthew bishop iv</t>
+          <t>ronald b russell</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -16127,11 +16127,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
-        <v>18529.56</v>
+        <v>22582.5</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -16142,7 +16142,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ronald b russell</t>
+          <t>steven matthew bishop iv</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -16155,11 +16155,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>16312.5</v>
+        <v>19079.56</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -16327,7 +16327,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>8332.709999999999</v>
+        <v>10297.71</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17363,7 +17363,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5701.02</v>
+        <v>6676.02</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17461,7 +17461,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1000.71</v>
+        <v>1001.4</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17741,7 +17741,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>8050</v>
+        <v>10300</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17867,7 +17867,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3284.51</v>
+        <v>3784.51</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17965,7 +17965,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3565</v>
+        <v>3569.1</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17993,7 +17993,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1650</v>
+        <v>1894.24</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -18063,7 +18063,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2950</v>
+        <v>3475</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18133,7 +18133,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>18731.79</v>
+        <v>21181.79</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18231,7 +18231,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2700.66</v>
+        <v>5025.66</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18329,7 +18329,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>18002.47</v>
+        <v>18527.47</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18427,7 +18427,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1835</v>
+        <v>1985</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18623,7 +18623,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>40305.24</v>
+        <v>41505.24</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18721,7 +18721,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3637.56</v>
+        <v>4937.56</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18847,7 +18847,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4850</v>
+        <v>5750</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19015,7 +19015,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1410</v>
+        <v>4600</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19113,7 +19113,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3760</v>
+        <v>5294.87</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19337,7 +19337,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2673.46</v>
+        <v>4353.16</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19435,7 +19435,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>15007.15</v>
+        <v>17052.15</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19463,7 +19463,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>6856.01</v>
+        <v>9576.01</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -19589,7 +19589,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>13942.27</v>
+        <v>20588.27</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19715,7 +19715,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>27794</v>
+        <v>29909</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19743,7 +19743,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>5969.95</v>
+        <v>6664.95</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>

</xml_diff>